<commit_message>
Mejora de notas Eliminacion de funciones en desuso Actualizacion de datos tras extraccion con eliminacion de alternativas repetidas mas estricta, sin modelos repetidos
</commit_message>
<xml_diff>
--- a/data/data_preparation/smartband/df_relation_matrix.xlsx
+++ b/data/data_preparation/smartband/df_relation_matrix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,39 +446,39 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Capacidad de la batería</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Duración de la batería</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tamaño de la pantalla</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo de pantalla</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Es resistente al agua</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Capacidad de la batería</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Duración de la batería</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Tamaño de la pantalla</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo de pantalla</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Resolución máxima</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Con pantalla táctil</t>
@@ -486,20 +486,15 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Es resistente al agua</t>
+          <t>funciones</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>funciones</t>
+          <t>facil</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>facil</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>conecta</t>
         </is>
@@ -550,9 +545,6 @@
       <c r="N2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -567,16 +559,16 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -597,9 +589,6 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -640,15 +629,12 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -692,12 +678,9 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -720,19 +703,19 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
         <v>1</v>
@@ -744,9 +727,6 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -793,9 +773,6 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -812,39 +789,36 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>3</v>
       </c>
-      <c r="E8" t="n">
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>